<commit_message>
fix: résolution du timeout Lambda lié à la connexion MySQL
</commit_message>
<xml_diff>
--- a/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Feuille de calcul de la base de connaissance-1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soni-info Tech\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ODC-AWS\ProjetFilRouge\ProjetHTML\Portfolio_Siakha_KABA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B0CF897-EB01-4766-A35F-6FDFD6F844CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E8DD12-542D-42EA-95B6-D2D20E0ED314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="55">
   <si>
     <t>Commentaires</t>
   </si>
@@ -287,12 +287,33 @@
   <si>
     <t>Ex 5</t>
   </si>
+  <si>
+    <t>Réseau / Configuration AWS (fonction Lambda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Échec de connexion entre la fonction AWS Lambda et la base de données MySQL hébergée sur une instance EC2. </t>
+  </si>
+  <si>
+    <t>Message d’erreur “Task timed out after 3.00 seconds”, absence de réponse de la base de données, exécution interrompue après 3 secondes</t>
+  </si>
+  <si>
+    <t>Le port 3306 (port MySQL) n’est pas autorisé dans les règles du groupe de sécurité de l’instance EC2, ce qui bloque la communication entre Lambda et la base de données.</t>
+  </si>
+  <si>
+    <t>Ajouter une règle entrante dans le groupe de sécurité de l’EC2 pour autoriser le port 3306 et permettre l’accès depuis la fonction Lambda (ou son groupe de sécurité).</t>
+  </si>
+  <si>
+    <t>Console AWS (EC2, VPC, Security Groups)</t>
+  </si>
+  <si>
+    <t>exemple 5</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -383,6 +404,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Amazon Ember"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -415,7 +442,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -438,106 +465,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -551,15 +484,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -572,40 +496,25 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -947,167 +856,191 @@
     <col min="10" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="11" customFormat="1" ht="65.400000000000006" customHeight="1" thickBot="1">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:9" s="8" customFormat="1" ht="65.400000000000006" customHeight="1">
+      <c r="A1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="10"/>
+      <c r="I1" s="7"/>
     </row>
     <row r="2" spans="1:9" ht="409.2" customHeight="1">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="14" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="279.89999999999998" customHeight="1">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="14" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="207" customHeight="1">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="207" customHeight="1" thickBot="1">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:9" ht="207" customHeight="1">
+      <c r="A5" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="14" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="49.95" customHeight="1">
+    <row r="6" spans="1:9" ht="199.95" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="49.95" customHeight="1">
+      <c r="B6" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="100.05" customHeight="1">
       <c r="A7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="49.95" customHeight="1">
+    <row r="8" spans="1:9" ht="100.05" customHeight="1">
       <c r="A8" s="4"/>
     </row>
-    <row r="9" spans="1:9" ht="49.95" customHeight="1">
+    <row r="9" spans="1:9" ht="100.05" customHeight="1">
       <c r="A9" s="4"/>
     </row>
-    <row r="10" spans="1:9" ht="49.95" customHeight="1">
+    <row r="10" spans="1:9" ht="100.05" customHeight="1">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:9" ht="49.95" customHeight="1">
+    <row r="11" spans="1:9" ht="100.05" customHeight="1">
       <c r="A11" s="4"/>
     </row>
     <row r="12" spans="1:9" ht="49.95" customHeight="1">
@@ -1724,6 +1657,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -1946,12 +1885,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
@@ -1961,6 +1894,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9479F6B-BC70-40D1-9DD0-21D0DC99C2BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1977,21 +1927,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9479F6B-BC70-40D1-9DD0-21D0DC99C2BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(Lab-173) : correction de l’erreur AMI et du port HTTP dans le script EC2
</commit_message>
<xml_diff>
--- a/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Feuille de calcul de la base de connaissance-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ODC-AWS\ProjetFilRouge\ProjetHTML\Portfolio_Siakha_KABA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E8DD12-542D-42EA-95B6-D2D20E0ED314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A159ADE2-4119-415C-8DE2-193C1B26A4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
   <si>
     <t>Commentaires</t>
   </si>
@@ -307,6 +307,64 @@
   </si>
   <si>
     <t>exemple 5</t>
+  </si>
+  <si>
+    <t>173--Lab - Résolution des problèmes de création d'instance</t>
+  </si>
+  <si>
+    <t>Problème 1</t>
+  </si>
+  <si>
+    <t>Problème 2</t>
+  </si>
+  <si>
+    <t>Déploiement EC2 / AMI</t>
+  </si>
+  <si>
+    <t>L’instance EC2 ne peut pas être lancée car l’ID de l’image (AMI) est introuvable</t>
+  </si>
+  <si>
+    <t>Erreur : InvalidAMIID.NotFound lors de l’exécution de la commande run-instances</t>
+  </si>
+  <si>
+    <t>L’AMI utilisée n’existe pas dans la région où l’instance est lancée. Dans le script, l’AMI est récupérée avec --region $region ou us-west-2 mais l’instance est lancée avec --region us-east-1, ce qui crée une incohérence</t>
+  </si>
+  <si>
+    <t>Vérifier la région utilisée dans run-instances
+Remplacer us-east-1 par $region ou us-west-2 dans le script
+Vérifier que l’AMI existe dans la région avec describe-images
+Relancer le script après correction</t>
+  </si>
+  <si>
+    <t>AWS CLI (describe-images, run-instances)</t>
+  </si>
+  <si>
+    <t>Les AMI sont spécifiques à chaque région AWS. Une incohérence de région est une cause fréquente de cette erreur</t>
+  </si>
+  <si>
+    <t>Réseau / Service Web</t>
+  </si>
+  <si>
+    <t>L’instance EC2 est lancée mais la page web ne s’affiche pas</t>
+  </si>
+  <si>
+    <t>Impossible d’accéder à http://&lt;public-ip&gt;</t>
+  </si>
+  <si>
+    <t>Port 80 fermé
+- Serveur web (httpd) non démarré
+- Mauvaise configuration du groupe de sécurté</t>
+  </si>
+  <si>
+    <t>Vérifier le Security Group → autoriser HTTP (port 80)
+- Se connecter via EC2 Instance Connect</t>
+  </si>
+  <si>
+    <t>EC2 Instance Connect
+Security Groups AWS</t>
+  </si>
+  <si>
+    <t>Problème  fréquent après déploiement si le serveur web n’est pas actif ou si le port est bloqué</t>
   </si>
 </sst>
 </file>
@@ -499,22 +557,22 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1028,11 +1086,63 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="100.05" customHeight="1">
-      <c r="A7" s="4"/>
-    </row>
-    <row r="8" spans="1:9" ht="100.05" customHeight="1">
-      <c r="A8" s="4"/>
+    <row r="7" spans="1:9" ht="250.05" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="250.05" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="100.05" customHeight="1">
       <c r="A9" s="4"/>
@@ -1585,7 +1695,7 @@
   </sheetData>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B5 B7:B1048576" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B5 B9:B1048576" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
   </dataValidations>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="10" orientation="landscape" horizontalDpi="4294967293" verticalDpi="1200" r:id="rId1"/>
@@ -1657,12 +1767,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -1885,6 +1989,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
@@ -1894,23 +2004,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9479F6B-BC70-40D1-9DD0-21D0DC99C2BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1927,4 +2020,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9479F6B-BC70-40D1-9DD0-21D0DC99C2BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix: correction des problèmes de connectivité VPC en ajoutant la route vers l’Internet Gateway et en supprimant la règle NACL bloquant le SSH
</commit_message>
<xml_diff>
--- a/Feuille de calcul de la base de connaissance-1.xlsx
+++ b/Feuille de calcul de la base de connaissance-1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr showInkAnnotation="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ODC-AWS\ProjetFilRouge\ProjetHTML\Portfolio_Siakha_KABA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A159ADE2-4119-415C-8DE2-193C1B26A4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC80A9C8-1518-418A-AA9A-85F655626712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="88">
   <si>
     <t>Commentaires</t>
   </si>
@@ -365,6 +365,61 @@
   </si>
   <si>
     <t>Problème  fréquent après déploiement si le serveur web n’est pas actif ou si le port est bloqué</t>
+  </si>
+  <si>
+    <t>Réseau (Routing / Internet Access)</t>
+  </si>
+  <si>
+    <t>Le serveur web n’est pas accessible depuis Internet</t>
+  </si>
+  <si>
+    <t>Page web inaccessible
+- Timeout navigateur
+- Aucun port détecté avec nmap</t>
+  </si>
+  <si>
+    <t>Absence de route par défaut (0.0.0.0/0) vers l’Internet Gateway dans la table de routage du sous-réseau public</t>
+  </si>
+  <si>
+    <t>Vérifier la table de routage
+- Ajouter une route vers Internet Gateway</t>
+  </si>
+  <si>
+    <t>Problème classique : un subnet “public” sans route IGW n’est pas réellement public</t>
+  </si>
+  <si>
+    <t>Problème 3</t>
+  </si>
+  <si>
+    <t>Problème 4</t>
+  </si>
+  <si>
+    <t>Sécurité réseau (NACL)</t>
+  </si>
+  <si>
+    <t>Impossible de se connecter en SSH malgré un Security Group correct</t>
+  </si>
+  <si>
+    <t>Échec connexion EC2 Instance Connect
+- SSH timeout
+- Port 22 ouvert mais inaccessible</t>
+  </si>
+  <si>
+    <t>Une règle NACL bloque le trafic entrant ou sortant sur le port 22</t>
+  </si>
+  <si>
+    <t>Vérifier les Network ACL
+- Supprimer la règle bloquante</t>
+  </si>
+  <si>
+    <t>AWS CLI 
+ Flow Logs VPC</t>
+  </si>
+  <si>
+    <t>Piège fréquent : NACL = stateless → nécessite autorisation entrée + sortie</t>
+  </si>
+  <si>
+    <t>181--Lab - Dépanner un VPC</t>
   </si>
 </sst>
 </file>
@@ -1144,11 +1199,60 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="100.05" customHeight="1">
-      <c r="A9" s="4"/>
-    </row>
-    <row r="10" spans="1:9" ht="100.05" customHeight="1">
-      <c r="A10" s="4"/>
+    <row r="9" spans="1:9" ht="199.95" customHeight="1">
+      <c r="A9" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="199.95" customHeight="1">
+      <c r="A10" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="100.05" customHeight="1">
       <c r="A11" s="4"/>
@@ -1767,6 +1871,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -1989,12 +2099,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
@@ -2004,6 +2108,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9479F6B-BC70-40D1-9DD0-21D0DC99C2BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2020,21 +2141,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9479F6B-BC70-40D1-9DD0-21D0DC99C2BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>